<commit_message>
feat(app): a fila ganha linha nova, e o Cliente passa a escrever no mapa
- ausencia de preenchimento deixa de ser cor desconhecida: sem isso toda linha criada iria para a quarentena
- PendingRowInsert na fila, sem sourceRow e sem previous, com a defesa oposta: a REF nao pode existir
- a ancora vem das linhas CRUAS, com piso em firstDataRow, senao a gravacao caia no cabecalho
- PUT /api/processes/:ref/client grava a regra de consolidacao e cria o arquivo se faltar, que e o estado de PD-08
- a fixture ganha cor real fora do mapa, para a quarentena por cor nao ficar sem prova
</commit_message>
<xml_diff>
--- a/tests/fixtures/cores.xlsx
+++ b/tests/fixtures/cores.xlsx
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
   <si>
     <t>REF</t>
   </si>
@@ -174,6 +174,12 @@
   </si>
   <si>
     <t>COR DESCONHECIDA</t>
+  </si>
+  <si>
+    <t>FT998.26</t>
+  </si>
+  <si>
+    <t>SEM COR</t>
   </si>
 </sst>
 </file>
@@ -2996,7 +3002,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFB5C4C1-7B16-415C-9319-3F9A3F1843AE}">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr defaultRowHeight="31.5" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="12.140625" style="162" bestFit="1" customWidth="1"/>
@@ -3176,16 +3182,28 @@
       <c r="L10" s="281"/>
     </row>
     <row r="11" spans="1:16">
-      <c r="A11" s="163" t="s">
+      <c r="A11" s="169" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="163" t="s">
+      <c r="B11" s="169" t="s">
         <v>35</v>
       </c>
-      <c r="I11" s="163">
+      <c r="I11" s="169">
         <v>46244</v>
       </c>
-      <c r="L11" s="163"/>
+      <c r="L11" s="169"/>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12" s="163" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="163" t="s">
+        <v>37</v>
+      </c>
+      <c r="I12" s="163">
+        <v>46244</v>
+      </c>
+      <c r="L12" s="163"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>